<commit_message>
resultado actualizado carga ob fixed 3 estaciones
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH/Carga_on_board_fixed_1estacion/elmo_data.xlsx
+++ b/data/Escenarios_DCH/Carga_on_board_fixed_1estacion/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH\Carga_on_board_fixed_1estacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D77E6C9-1741-4370-9B5E-EB983EFDD20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB78CE51-ED37-419C-A27A-036D7BEEEEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -3382,7 +3382,7 @@
   <cols>
     <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3465,6 +3465,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>